<commit_message>
Replace inherited frame with shell-first barrel and structural hatch
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="1" r:id="R9a182243ad194ec2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="1" r:id="R1fd211c12b8c434d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -174,8 +174,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RollerBOM" displayName="RollerBOM" ref="A9:O41" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A9:O41"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RollerBOM" displayName="RollerBOM" ref="A9:O51" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A9:O51"/>
   <x:tableColumns count="15">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Part / exact model"/>
@@ -430,7 +430,7 @@
     </x:row>
     <x:row r="2" ht="29" customHeight="1">
       <x:c r="A2" s="5" t="str">
-        <x:v>Owned INJORA INJS035-360 locked. ONE reusable vehicle drive end section. No new servo/programmer purchase. Powered release held.</x:v>
+        <x:v>Owned INJORA INJS035-360 locked. Complete shell and hatch with ONE populated drive. No new servo/programmer purchase. Powered release held.</x:v>
       </x:c>
       <x:c r="B2" s="5"/>
       <x:c r="C2" s="5"/>
@@ -455,8 +455,8 @@
       <x:c r="C3" s="7"/>
       <x:c r="D3" s="7"/>
       <x:c r="E3" s="9" t="n">
-        <x:f>SUM(K10:K41)</x:f>
-        <x:v>33.040000000000006</x:v>
+        <x:f>SUM(K10:K51)</x:f>
+        <x:v>35.720000000000006</x:v>
       </x:c>
       <x:c r="F3" s="1" t="str">
         <x:v>USD; excludes tax, delivery, shaft preparation and every blank-price / HOLD item. This is not a vehicle total.</x:v>
@@ -805,7 +805,7 @@
         <x:v>2026-09-13</x:v>
       </x:c>
       <x:c r="N13" s="13" t="str">
-        <x:v>Four each drive side. Confirm actual fit/drag on coupon; not a load rating.</x:v>
+        <x:v>Four each drive side. Confirm actual fit/drag on coupon; not a load rating. Purchased 608 batch must be checked against split seat and inner-race spacer contact.</x:v>
       </x:c>
       <x:c r="O13" s="13" t="str">
         <x:v>Support</x:v>
@@ -855,7 +855,7 @@
         <x:v>2026-09-13</x:v>
       </x:c>
       <x:c r="N14" s="13" t="str">
-        <x:v>16 mm square M4 pattern;22.5 overall axial envelope,30.6 circumscribed diameter.</x:v>
+        <x:v>16 mm square M4 pattern;22.5 overall axial envelope,30.6 circumscribed diameter. Hub clamps shaft and retains outboard bearing inner race through0.5 shim plus10 spacer; confirm rated clamp torque and measured endplay.</x:v>
       </x:c>
       <x:c r="O14" s="13" t="str">
         <x:v>Support</x:v>
@@ -873,10 +873,10 @@
         <x:v>BUY ONE SIDE</x:v>
       </x:c>
       <x:c r="D15" s="15" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E15" s="15" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F15" s="15" t="n">
         <x:v>0</x:v>
@@ -886,7 +886,7 @@
       </x:c>
       <x:c r="H15" s="15" t="n">
         <x:f>IF(E15=0,0,MAX(E15-F15-G15,0))</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I15" s="15" t="n">
         <x:v>1</x:v>
@@ -896,7 +896,7 @@
       </x:c>
       <x:c r="K15" s="17" t="n">
         <x:f>IF(H15=0,0,IF(ISNUMBER(J15),ROUNDUP(H15/I15,0)*J15,""))</x:f>
-        <x:v>9.98</x:v>
+        <x:v>4.99</x:v>
       </x:c>
       <x:c r="L15" s="18" t="str">
         <x:v>https://www.gobilda.com/2910-series-aluminum-clamping-collar-8mm-id-x-21mm-od-9mm-length/</x:v>
@@ -905,7 +905,7 @@
         <x:v>2026-09-13</x:v>
       </x:c>
       <x:c r="N15" s="13" t="str">
-        <x:v>Two per wheel shaft; input retention separate and unresolved. Actual9 mm length.</x:v>
+        <x:v>One inboard collar per drive, moved inward3 mm. Clamping wheel hub supplies outboard retention through purchased metal spacers/shim. Verify endplay without bearing preload.</x:v>
       </x:c>
       <x:c r="O15" s="13" t="str">
         <x:v>Support</x:v>
@@ -955,7 +955,7 @@
         <x:v>2026-09-13</x:v>
       </x:c>
       <x:c r="N16" s="13" t="str">
-        <x:v>150 mm blank needs110 mm finished length and clutch flat. Verify purchased finish/fit and local cutting or order prepared shafts; no workshop assumed.</x:v>
+        <x:v>150 mm stock candidate cut to113 mm for revised wheel shaft; ends remain inside tire width. Ground journals, end finish and receiving dimensions HOLD.</x:v>
       </x:c>
       <x:c r="O16" s="13" t="str">
         <x:v>Support</x:v>
@@ -1001,7 +1001,7 @@
         <x:v>2026-09-13</x:v>
       </x:c>
       <x:c r="N17" s="13" t="str">
-        <x:v>49 mm shaft geometry Y55..104, with prepared end groove/retaining ring. Groove, shims, adapter and supplier remain HOLD; do not order a wrong specification.</x:v>
+        <x:v>Input bearing pair shifted 3 mm inward to Y70/96 on left, shaft envelope Y52..101; mirrored right. Prepared shaft length/end grooves and retention still HOLD.</x:v>
       </x:c>
       <x:c r="O17" s="13" t="str">
         <x:v>Support</x:v>
@@ -1199,16 +1199,16 @@
       </x:c>
       <x:c r="B22" s="13" t="str">
         <x:v>One complete 246 mm wheel print set
-P01 center + P02 bead ring + P03 TPU tread</x:v>
+230 mm rigid rim/web,246 mm only with provisional tread</x:v>
       </x:c>
       <x:c r="C22" s="13" t="str">
-        <x:v>DEFER WHEEL</x:v>
+        <x:v>HOLD WHEEL</x:v>
       </x:c>
       <x:c r="D22" s="15" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E22" s="15" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F22" s="15" t="n">
         <x:v>0</x:v>
@@ -1218,22 +1218,21 @@
       </x:c>
       <x:c r="H22" s="15" t="n">
         <x:f>IF(E22=0,0,MAX(E22-F22-G22,0))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I22" s="15" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J22" s="16"/>
-      <x:c r="K22" s="17" t="n">
+      <x:c r="K22" s="17" t="str">
         <x:f>IF(H22=0,0,IF(ISNUMBER(J22),ROUNDUP(H22/I22,0)*J22,""))</x:f>
-        <x:v>0</x:v>
       </x:c>
       <x:c r="L22" s="18" t="str"/>
       <x:c r="M22" s="19" t="str">
         <x:v>2026-09-13</x:v>
       </x:c>
       <x:c r="N22" s="13" t="str">
-        <x:v>Wheel/tire selection and printing deferred by user. Three STL parts; unpowered fit only. Offline X2D 0.4 mm slice estimates total 505 g filament / 20 h including print aids. Actual nozzle/material and physical fit unverified.</x:v>
+        <x:v>Imported wheel packaging retained; native hub holes added. Strength, mass reduction and tire/bead retention remain unqualified. Do not use archived bead hardware as current fit evidence. First clamped drive test omits tread; actual rolling radius must be used for later ground tests.</x:v>
       </x:c>
       <x:c r="O22" s="13" t="str">
         <x:v>Printed</x:v>
@@ -1244,17 +1243,17 @@
         <x:v>P03</x:v>
       </x:c>
       <x:c r="B23" s="13" t="str">
-        <x:v>Barrel, covers, lid, ribs and mounts
-D160x210</x:v>
+        <x:v>Single shell-first barrel housing and structural hatch
+Fresh native S02/S03 geometry; D160x210; no legacy frame</x:v>
       </x:c>
       <x:c r="C23" s="13" t="str">
-        <x:v>PRINT LATER</x:v>
+        <x:v>HOLD PRINT</x:v>
       </x:c>
       <x:c r="D23" s="15" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E23" s="15" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F23" s="15" t="n">
         <x:v>0</x:v>
@@ -1264,22 +1263,21 @@
       </x:c>
       <x:c r="H23" s="15" t="n">
         <x:f>IF(E23=0,0,MAX(E23-F23-G23,0))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I23" s="15" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J23" s="16"/>
-      <x:c r="K23" s="17" t="n">
+      <x:c r="K23" s="17" t="str">
         <x:f>IF(H23=0,0,IF(ISNUMBER(J23),ROUNDUP(H23/I23,0)*J23,""))</x:f>
-        <x:v>0</x:v>
       </x:c>
       <x:c r="L23" s="18" t="str"/>
       <x:c r="M23" s="19" t="str">
         <x:v>2026-09-13</x:v>
       </x:c>
       <x:c r="N23" s="13" t="str">
-        <x:v>Current end section uses D159 shell, D151 register and four M4 body mounts. Separate main drum and electronics lid remain later prints; do not duplicate the end section.</x:v>
+        <x:v>Final vehicle housing used for one populated drive bench test. Slicing, joint qualification, access and measured hardware gates apply.</x:v>
       </x:c>
       <x:c r="O23" s="13" t="str">
         <x:v>Printed</x:v>
@@ -1294,7 +1292,7 @@
 22.05/22.15/22.25 holes</x:v>
       </x:c>
       <x:c r="C24" s="13" t="str">
-        <x:v>PRINT GAUGE</x:v>
+        <x:v>HOLD GAUGE</x:v>
       </x:c>
       <x:c r="D24" s="15" t="n">
         <x:v>1</x:v>
@@ -1324,7 +1322,7 @@
         <x:v>2026-09-13</x:v>
       </x:c>
       <x:c r="N24" s="13" t="str">
-        <x:v>Non-powered PETG dimensional coupon,80x32x7; keep orientation consistent with final seats.</x:v>
+        <x:v>Historical22.05/22.15/22.25 bearing gauge brackets current22.2 trial bore. New shell nut/shoulder/strap coupon and print orientation still require preparation and validation.</x:v>
       </x:c>
       <x:c r="O24" s="13" t="str">
         <x:v>Printed</x:v>
@@ -1385,7 +1383,7 @@
 Consistent metric family</x:v>
       </x:c>
       <x:c r="C26" s="13" t="str">
-        <x:v>HOLD</x:v>
+        <x:v>HOLD REMAINDER</x:v>
       </x:c>
       <x:c r="D26" s="15"/>
       <x:c r="E26" s="15" t="n">
@@ -1412,7 +1410,7 @@
         <x:v>2026-09-13</x:v>
       </x:c>
       <x:c r="N26" s="13" t="str">
-        <x:v>Per drive: four M4 body bolts, eight M4 bearing-cap bolts and four M4 carriage bolts plus nuts/washers. Four M3 cover screws and four M3 saddle screws also required. Lengths/locking/tool fit remain to verify. Wheel hardware deferred separately.</x:v>
+        <x:v>Specific new housing fasteners itemized below. Remaining component restraints and washers still unresolved; no complete fastener kit claimed.</x:v>
       </x:c>
       <x:c r="O26" s="13" t="str">
         <x:v>Hardware</x:v>
@@ -1925,13 +1923,13 @@
 M4x10, ISO4762 / goBILDA2800-0004-0010</x:v>
       </x:c>
       <x:c r="C38" s="13" t="str">
-        <x:v>DEFER WHEEL</x:v>
+        <x:v>HOLD FIT</x:v>
       </x:c>
       <x:c r="D38" s="15" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E38" s="15" t="n">
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F38" s="15"/>
       <x:c r="G38" s="15" t="n">
@@ -1939,15 +1937,14 @@
       </x:c>
       <x:c r="H38" s="15" t="n">
         <x:f>IF(E38=0,0,MAX(E38-F38-G38,0))</x:f>
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I38" s="15" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J38" s="16"/>
-      <x:c r="K38" s="17" t="n">
+      <x:c r="K38" s="17" t="str">
         <x:f>IF(H38=0,0,IF(ISNUMBER(J38),ROUNDUP(H38/I38,0)*J38,""))</x:f>
-        <x:v>0</x:v>
       </x:c>
       <x:c r="L38" s="18" t="str">
         <x:v>https://www.gobilda.com/m4-socket-head-screws</x:v>
@@ -1956,7 +1953,7 @@
         <x:v>2026-09-13</x:v>
       </x:c>
       <x:c r="N38" s="13" t="str">
-        <x:v>Wheel/tire selection and printing deferred by user. Four per wheel. 5 mm nominal engagement with 5 mm web; verify actual hub and no bottoming. Price/pack choice pending.</x:v>
+        <x:v>Native wheel web has4x D4.4 holes on16 mm square. M4x10 gives nominal6 mm thread engagement through4 mm web; verify actual hub, head and tool access.</x:v>
       </x:c>
       <x:c r="O38" s="13" t="str">
         <x:v>Wheel hardware</x:v>
@@ -1971,10 +1968,10 @@
 M4x35 ISO4762; Accu SSC-M4-35-A2-R360 reference</x:v>
       </x:c>
       <x:c r="C39" s="13" t="str">
-        <x:v>DEFER WHEEL</x:v>
+        <x:v>HISTORICAL</x:v>
       </x:c>
       <x:c r="D39" s="15" t="n">
-        <x:v>16</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E39" s="15" t="n">
         <x:v>0</x:v>
@@ -2002,7 +1999,7 @@
         <x:v>2026-09-13</x:v>
       </x:c>
       <x:c r="N39" s="13" t="str">
-        <x:v>Wheel/tire selection and printing deferred by user. Eight per wheel. Nominal7 mm head diameter and4 mm height; head ends atY149.5, shaft tipY110.5. No washers in current stack. Pack/price unconfirmed.</x:v>
+        <x:v>Superseded three-piece wheel/bead concept; retained record only. No current purchase.</x:v>
       </x:c>
       <x:c r="O39" s="13" t="str">
         <x:v>Wheel hardware</x:v>
@@ -2017,10 +2014,10 @@
 M4x0.7 ISO4032 plain hex;7 mm AF,3.2 mm thickness reference</x:v>
       </x:c>
       <x:c r="C40" s="13" t="str">
-        <x:v>DEFER WHEEL</x:v>
+        <x:v>HISTORICAL</x:v>
       </x:c>
       <x:c r="D40" s="15" t="n">
-        <x:v>16</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E40" s="15" t="n">
         <x:v>0</x:v>
@@ -2046,7 +2043,7 @@
         <x:v>2026-09-13</x:v>
       </x:c>
       <x:c r="N40" s="13" t="str">
-        <x:v>Wheel/tire selection and printing deferred by user. Eight per wheel. Fit in7.3 mm AF pockets; verify nut lot dimensions. Mechanical witness marks for unpowered fit; locking method for operation remains to qualify.</x:v>
+        <x:v>Superseded three-piece wheel/bead concept; retained record only. No current purchase.</x:v>
       </x:c>
       <x:c r="O40" s="13" t="str">
         <x:v>Wheel hardware</x:v>
@@ -2057,11 +2054,11 @@
         <x:v>P06</x:v>
       </x:c>
       <x:c r="B41" s="13" t="str">
-        <x:v>Reusable vehicle drive end section + input spine
-drive-end-section.nbcad; PETG fit candidate</x:v>
+        <x:v>Removable input carriage and bearing-cap set
+Fresh native support parts; integral servo locating lips</x:v>
       </x:c>
       <x:c r="C41" s="13" t="str">
-        <x:v>FIT REVIEW</x:v>
+        <x:v>HOLD PRINT</x:v>
       </x:c>
       <x:c r="D41" s="15" t="n">
         <x:v>2</x:v>
@@ -2087,16 +2084,461 @@
         <x:f>IF(H41=0,0,IF(ISNUMBER(J41),ROUNDUP(H41/I41,0)*J41,""))</x:f>
       </x:c>
       <x:c r="L41" s="18" t="str">
-        <x:v>Local native CAD: drive-end-section.nbcad</x:v>
+        <x:v>Local native CAD: Roller-300.nbcad</x:v>
       </x:c>
       <x:c r="M41" s="19" t="str">
         <x:v>2026-09-13</x:v>
       </x:c>
       <x:c r="N41" s="13" t="str">
-        <x:v>Two structural meshes supplied for unpowered fit review after bearing coupon. Same carrier clamps for testing and bolts to the drum. Caps/saddle/guard/shaft interfaces still need completion before a powered assembly.</x:v>
+        <x:v>Per side: input carriage, two wheel caps and two input caps. Old carrier/spine STLs are preserved historical fit candidates, not this test module.</x:v>
       </x:c>
       <x:c r="O41" s="13" t="str">
         <x:v>Printed drive</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="66" customHeight="1">
+      <x:c r="A42" s="13" t="str">
+        <x:v>H07</x:v>
+      </x:c>
+      <x:c r="B42" s="13" t="str">
+        <x:v>Structural hatch screws
+M4x12 countersunk 90deg candidate</x:v>
+      </x:c>
+      <x:c r="C42" s="13" t="str">
+        <x:v>HOLD FIT</x:v>
+      </x:c>
+      <x:c r="D42" s="15" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E42" s="15" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F42" s="15"/>
+      <x:c r="G42" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H42" s="15" t="n">
+        <x:f>IF(E42=0,0,MAX(E42-F42-G42,0))</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I42" s="15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J42" s="16"/>
+      <x:c r="K42" s="17" t="str">
+        <x:f>IF(H42=0,0,IF(ISNUMBER(J42),ROUNDUP(H42/I42,0)*J42,""))</x:f>
+      </x:c>
+      <x:c r="L42" s="18"/>
+      <x:c r="M42" s="19" t="str">
+        <x:v>2026-09-19</x:v>
+      </x:c>
+      <x:c r="N42" s="13" t="str">
+        <x:v>Eight radial hatch fasteners. Verify actual head diameter, seating and preload; price/source unselected.</x:v>
+      </x:c>
+      <x:c r="O42" s="13" t="str">
+        <x:v>Shell fasteners</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="66" customHeight="1">
+      <x:c r="A43" s="13" t="str">
+        <x:v>H08</x:v>
+      </x:c>
+      <x:c r="B43" s="13" t="str">
+        <x:v>Wheel bearing-cap screws
+M4x35 socket-head candidate</x:v>
+      </x:c>
+      <x:c r="C43" s="13" t="str">
+        <x:v>HOLD FIT</x:v>
+      </x:c>
+      <x:c r="D43" s="15" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E43" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F43" s="15"/>
+      <x:c r="G43" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H43" s="15" t="n">
+        <x:f>IF(E43=0,0,MAX(E43-F43-G43,0))</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I43" s="15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J43" s="16"/>
+      <x:c r="K43" s="17" t="str">
+        <x:f>IF(H43=0,0,IF(ISNUMBER(J43),ROUNDUP(H43/I43,0)*J43,""))</x:f>
+      </x:c>
+      <x:c r="L43" s="18"/>
+      <x:c r="M43" s="19" t="str">
+        <x:v>2026-09-19</x:v>
+      </x:c>
+      <x:c r="N43" s="13" t="str">
+        <x:v>Two per wheel cap; four caps vehicle, two first drive. Tool reach and actual thread engagement require fit check.</x:v>
+      </x:c>
+      <x:c r="O43" s="13" t="str">
+        <x:v>Shell fasteners</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="66" customHeight="1">
+      <x:c r="A44" s="13" t="str">
+        <x:v>H09</x:v>
+      </x:c>
+      <x:c r="B44" s="13" t="str">
+        <x:v>Carriage tension screws
+M4x12 socket-head candidate</x:v>
+      </x:c>
+      <x:c r="C44" s="13" t="str">
+        <x:v>HOLD FIT</x:v>
+      </x:c>
+      <x:c r="D44" s="15" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E44" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F44" s="15"/>
+      <x:c r="G44" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H44" s="15" t="n">
+        <x:f>IF(E44=0,0,MAX(E44-F44-G44,0))</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I44" s="15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J44" s="16"/>
+      <x:c r="K44" s="17" t="str">
+        <x:f>IF(H44=0,0,IF(ISNUMBER(J44),ROUNDUP(H44/I44,0)*J44,""))</x:f>
+      </x:c>
+      <x:c r="L44" s="18"/>
+      <x:c r="M44" s="19" t="str">
+        <x:v>2026-09-19</x:v>
+      </x:c>
+      <x:c r="N44" s="13" t="str">
+        <x:v>Four per carriage with sliding slots. Check washers/head clearance and locking.</x:v>
+      </x:c>
+      <x:c r="O44" s="13" t="str">
+        <x:v>Shell fasteners</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="66" customHeight="1">
+      <x:c r="A45" s="13" t="str">
+        <x:v>H10</x:v>
+      </x:c>
+      <x:c r="B45" s="13" t="str">
+        <x:v>Input bearing-cap screws
+M3x30 socket-head candidate</x:v>
+      </x:c>
+      <x:c r="C45" s="13" t="str">
+        <x:v>HOLD FIT</x:v>
+      </x:c>
+      <x:c r="D45" s="15" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E45" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F45" s="15"/>
+      <x:c r="G45" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H45" s="15" t="n">
+        <x:f>IF(E45=0,0,MAX(E45-F45-G45,0))</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I45" s="15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J45" s="16"/>
+      <x:c r="K45" s="17" t="str">
+        <x:f>IF(H45=0,0,IF(ISNUMBER(J45),ROUNDUP(H45/I45,0)*J45,""))</x:f>
+      </x:c>
+      <x:c r="L45" s="18"/>
+      <x:c r="M45" s="19" t="str">
+        <x:v>2026-09-19</x:v>
+      </x:c>
+      <x:c r="N45" s="13" t="str">
+        <x:v>Head seats at Z137 in D6 counterbore; nominal headD5.5x3.0.30 mm screw extends to Z107 through nut pocket109..111.8. Verify received fastener and printed fit.</x:v>
+      </x:c>
+      <x:c r="O45" s="13" t="str">
+        <x:v>Shell fasteners</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="66" customHeight="1">
+      <x:c r="A46" s="13" t="str">
+        <x:v>H11</x:v>
+      </x:c>
+      <x:c r="B46" s="13" t="str">
+        <x:v>Input-cap captive hex nuts
+M3 hex;5.5 mm AF reference</x:v>
+      </x:c>
+      <x:c r="C46" s="13" t="str">
+        <x:v>HOLD FIT</x:v>
+      </x:c>
+      <x:c r="D46" s="15" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E46" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F46" s="15"/>
+      <x:c r="G46" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H46" s="15" t="n">
+        <x:f>IF(E46=0,0,MAX(E46-F46-G46,0))</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I46" s="15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J46" s="16"/>
+      <x:c r="K46" s="17" t="str">
+        <x:f>IF(H46=0,0,IF(ISNUMBER(J46),ROUNDUP(H46/I46,0)*J46,""))</x:f>
+      </x:c>
+      <x:c r="L46" s="18"/>
+      <x:c r="M46" s="19" t="str">
+        <x:v>2026-09-19</x:v>
+      </x:c>
+      <x:c r="N46" s="13" t="str">
+        <x:v>Pocket width5.8, depth2.8; received nut and printed coupon verification required.</x:v>
+      </x:c>
+      <x:c r="O46" s="13" t="str">
+        <x:v>Shell fasteners</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="66" customHeight="1">
+      <x:c r="A47" s="13" t="str">
+        <x:v>H12</x:v>
+      </x:c>
+      <x:c r="B47" s="13" t="str">
+        <x:v>Housing captive hex nuts
+M4 hex;7 mm AF,3.2 mm reference</x:v>
+      </x:c>
+      <x:c r="C47" s="13" t="str">
+        <x:v>HOLD FIT</x:v>
+      </x:c>
+      <x:c r="D47" s="15" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="E47" s="15" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F47" s="15"/>
+      <x:c r="G47" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H47" s="15" t="n">
+        <x:f>IF(E47=0,0,MAX(E47-F47-G47,0))</x:f>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="I47" s="15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J47" s="16"/>
+      <x:c r="K47" s="17" t="str">
+        <x:f>IF(H47=0,0,IF(ISNUMBER(J47),ROUNDUP(H47/I47,0)*J47,""))</x:f>
+      </x:c>
+      <x:c r="L47" s="18"/>
+      <x:c r="M47" s="19" t="str">
+        <x:v>2026-09-19</x:v>
+      </x:c>
+      <x:c r="N47" s="13" t="str">
+        <x:v>Hatch8 + wheel caps8 + carriage8 vehicle; first populated side uses16. Nominal pockets7.3 AF /3.5 thick; check insertion and rotation restraint.</x:v>
+      </x:c>
+      <x:c r="O47" s="13" t="str">
+        <x:v>Shell fasteners</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="66" customHeight="1">
+      <x:c r="A48" s="13" t="str">
+        <x:v>M12</x:v>
+      </x:c>
+      <x:c r="B48" s="13" t="str">
+        <x:v>Inboard bearing inner-race spacer
+1522-0010-0030;8 ID x10 OD x3 mm</x:v>
+      </x:c>
+      <x:c r="C48" s="13" t="str">
+        <x:v>BUY FIT CHECK</x:v>
+      </x:c>
+      <x:c r="D48" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E48" s="15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F48" s="15"/>
+      <x:c r="G48" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H48" s="15" t="n">
+        <x:f>IF(E48=0,0,MAX(E48-F48-G48,0))</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I48" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J48" s="16" t="n">
+        <x:v>2.99</x:v>
+      </x:c>
+      <x:c r="K48" s="17" t="n">
+        <x:f>IF(H48=0,0,IF(ISNUMBER(J48),ROUNDUP(H48/I48,0)*J48,""))</x:f>
+        <x:v>2.99</x:v>
+      </x:c>
+      <x:c r="L48" s="18" t="str">
+        <x:v>https://www.gobilda.com/1522-series-8mm-id-spacer-10mm-od-3mm-length-4-pack/</x:v>
+      </x:c>
+      <x:c r="M48" s="19" t="str">
+        <x:v>2026-09-19</x:v>
+      </x:c>
+      <x:c r="N48" s="13" t="str">
+        <x:v>Published nominal dimensions; steel0.62 g each. Received tolerance and endplay verification remain. Price observed, stock/delivery not guaranteed; no purchase made.</x:v>
+      </x:c>
+      <x:c r="O48" s="13" t="str">
+        <x:v>Wheel retention</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="66" customHeight="1">
+      <x:c r="A49" s="13" t="str">
+        <x:v>M13</x:v>
+      </x:c>
+      <x:c r="B49" s="13" t="str">
+        <x:v>Outboard wheel retention spacer
+1529-0012-0100;8 ID x12 OD x10 mm</x:v>
+      </x:c>
+      <x:c r="C49" s="13" t="str">
+        <x:v>BUY FIT CHECK</x:v>
+      </x:c>
+      <x:c r="D49" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E49" s="15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F49" s="15"/>
+      <x:c r="G49" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H49" s="15" t="n">
+        <x:f>IF(E49=0,0,MAX(E49-F49-G49,0))</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I49" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J49" s="16" t="n">
+        <x:v>1.99</x:v>
+      </x:c>
+      <x:c r="K49" s="17" t="n">
+        <x:f>IF(H49=0,0,IF(ISNUMBER(J49),ROUNDUP(H49/I49,0)*J49,""))</x:f>
+        <x:v>1.99</x:v>
+      </x:c>
+      <x:c r="L49" s="18" t="str">
+        <x:v>https://www.gobilda.com/8mm-id-steel-spacer-12mm-od-10mm-length-4-pack/</x:v>
+      </x:c>
+      <x:c r="M49" s="19" t="str">
+        <x:v>2026-09-19</x:v>
+      </x:c>
+      <x:c r="N49" s="13" t="str">
+        <x:v>Published nominal dimensions;4.8 g each.0.5 mm shim sits against bearing; spacer extends to hub. Price observed, stock/delivery not guaranteed; no purchase made.</x:v>
+      </x:c>
+      <x:c r="O49" s="13" t="str">
+        <x:v>Wheel retention</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="66" customHeight="1">
+      <x:c r="A50" s="13" t="str">
+        <x:v>M14</x:v>
+      </x:c>
+      <x:c r="B50" s="13" t="str">
+        <x:v>Outboard inner-race shim
+2807-0811-0500;8 ID x11 OD x0.5 mm</x:v>
+      </x:c>
+      <x:c r="C50" s="13" t="str">
+        <x:v>BUY FIT CHECK</x:v>
+      </x:c>
+      <x:c r="D50" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E50" s="15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F50" s="15"/>
+      <x:c r="G50" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H50" s="15" t="n">
+        <x:f>IF(E50=0,0,MAX(E50-F50-G50,0))</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I50" s="15" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="J50" s="16" t="n">
+        <x:v>2.69</x:v>
+      </x:c>
+      <x:c r="K50" s="17" t="n">
+        <x:f>IF(H50=0,0,IF(ISNUMBER(J50),ROUNDUP(H50/I50,0)*J50,""))</x:f>
+        <x:v>2.69</x:v>
+      </x:c>
+      <x:c r="L50" s="18" t="str">
+        <x:v>https://www.gobilda.com/2807-series-stainless-steel-shim-8mm-id-x-11mm-od-0-50mm-thickness-12-pack/</x:v>
+      </x:c>
+      <x:c r="M50" s="19" t="str">
+        <x:v>2026-09-19</x:v>
+      </x:c>
+      <x:c r="N50" s="13" t="str">
+        <x:v>Published nominal dimensions; stainless steel0.18 g each. Confirm inner-race-only contact and endplay. Price observed, stock/delivery not guaranteed; no purchase made.</x:v>
+      </x:c>
+      <x:c r="O50" s="13" t="str">
+        <x:v>Wheel retention</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="66" customHeight="1">
+      <x:c r="A51" s="13" t="str">
+        <x:v>H13</x:v>
+      </x:c>
+      <x:c r="B51" s="13" t="str">
+        <x:v>Removable servo restraint straps
+8 mm width candidate; length measured after horn/ear check</x:v>
+      </x:c>
+      <x:c r="C51" s="13" t="str">
+        <x:v>HOLD FIT</x:v>
+      </x:c>
+      <x:c r="D51" s="15" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E51" s="15" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F51" s="15"/>
+      <x:c r="G51" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H51" s="15" t="n">
+        <x:f>IF(E51=0,0,MAX(E51-F51-G51,0))</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I51" s="15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J51" s="16"/>
+      <x:c r="K51" s="17" t="str">
+        <x:f>IF(H51=0,0,IF(ISNUMBER(J51),ROUNDUP(H51/I51,0)*J51,""))</x:f>
+      </x:c>
+      <x:c r="L51" s="18"/>
+      <x:c r="M51" s="19" t="str">
+        <x:v>2026-09-19</x:v>
+      </x:c>
+      <x:c r="N51" s="13" t="str">
+        <x:v>Two straps per servo through native2x8 mm carriage passages. Not a substitute for verified torque reaction/positive mount.</x:v>
+      </x:c>
+      <x:c r="O51" s="13" t="str">
+        <x:v>Shell fasteners</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2110,20 +2552,20 @@
     <x:mergeCell ref="A6:O6"/>
     <x:mergeCell ref="A7:O7"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="C10:C41">
+  <x:conditionalFormatting sqref="C10:C51">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="HOLD"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="BUY"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="OWNED"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="whole" operator="between" sqref="E10:G41">
+    <x:dataValidation type="whole" operator="between" sqref="E10:G51">
       <x:formula1>0</x:formula1>
       <x:formula2>1000</x:formula2>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23a2c94565e6429f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc54a61c4aa3748d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>